<commit_message>
feat: version 2.32.0 - modelo de suscripciones premium, micro-consejos IA con cache local, optimizaciones multiperfil y actualizacion documental
</commit_message>
<xml_diff>
--- a/documentos/Cronograma_de_Actividades_MediTime_Actualizado.xlsx
+++ b/documentos/Cronograma_de_Actividades_MediTime_Actualizado.xlsx
@@ -663,7 +663,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A2:V27"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="64" customWidth="1" min="2" max="2"/>
@@ -699,7 +699,7 @@
     <row r="3" ht="16" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Proyecto de Grado PGC (Noveno Semestre) — Vigencia 2026 | MediTime v2.31.1</t>
+          <t>Proyecto de Grado PGC (Noveno Semestre) — Vigencia 2026 | MediTime v2.32.0</t>
         </is>
       </c>
     </row>
@@ -1490,7 +1490,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A2:V26"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="66" customWidth="1" min="2" max="2"/>
@@ -1526,7 +1526,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Visión Macro-Evolutiva Anual (Febrero – Noviembre 2026) | MediTime v2.31.1</t>
+          <t>Visión Macro-Evolutiva Anual (Febrero – Noviembre 2026) | MediTime v2.32.0</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A2:F13"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="38" customWidth="1" min="2" max="2"/>

</xml_diff>